<commit_message>
Add baseline-safe profile and My Menu impact workflow
</commit_message>
<xml_diff>
--- a/docs/downloads/Subject Settings Matrix.xlsx
+++ b/docs/downloads/Subject Settings Matrix.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Subject Settings Matrix" sheetId="1" r:id="R824ee18e150241cb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="C1-C3 Defaults" sheetId="2" r:id="R28d78cec9aee4da1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Subject Settings Matrix" sheetId="1" r:id="R2afe67f6ee2840ff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="C1-C3 Defaults" sheetId="2" r:id="R14fd38c3c264479f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -442,13 +442,13 @@
     <xdr:ext cx="24765000" cy="1200150"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="576ca5da-cf47-4658-9a49-8a2d7b60f4c2"/>
+        <xdr:cNvPr id="1" name="054b8a2c-517e-4233-a27b-2ea6128ec031"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R1df47e7eae0a4738"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R6443544de43e4be6"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3564,9 +3564,9 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing ns1:id="R067a38a0f2224c49"/>
+  <x:drawing ns1:id="R88e47254ab084a2f"/>
   <x:tableParts count="1">
-    <x:tablePart ns1:id="Rf27bc0303c6045ae"/>
+    <x:tablePart ns1:id="Rd5a22c5ba6be4cab"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4169,7 +4169,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart ns1:id="Rbf3d86e136ad4681"/>
+    <x:tablePart ns1:id="R17fa0bab26a34961"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Organize cards for rapid camera setup
</commit_message>
<xml_diff>
--- a/docs/downloads/Subject Settings Matrix.xlsx
+++ b/docs/downloads/Subject Settings Matrix.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Subject Settings Matrix" sheetId="1" r:id="Re1db1ead78ab43e1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="C1-C3 Defaults" sheetId="2" r:id="R142c6c1c8fa1455c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Subject Settings Matrix" sheetId="1" r:id="R1605a80ff87a4e7b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="C1-C3 Defaults" sheetId="2" r:id="R300ecaccc8284d70"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -432,13 +432,13 @@
     <xdr:ext cx="24765000" cy="1200150"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="ebb6a567-5e25-4d25-b93e-b67911893025"/>
+        <xdr:cNvPr id="1" name="ef97ad79-dcc8-4f8a-bf02-5ad11eddf51a"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Re6a82793416b4b5e"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rf3c48f2783404676"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -5688,9 +5688,9 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing ns1:id="R3ad92f4855234330"/>
+  <x:drawing ns1:id="R3ce5f156e4b54536"/>
   <x:tableParts count="1">
-    <x:tablePart ns1:id="R2f45b775b8bc43cc"/>
+    <x:tablePart ns1:id="R2edb6d31fea54b68"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6812,7 +6812,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart ns1:id="Rf2514e0a8141408a"/>
+    <x:tablePart ns1:id="Rc8c04f183a464052"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Improve local apps and reconcile C1-C3 status
</commit_message>
<xml_diff>
--- a/docs/downloads/Subject Settings Matrix.xlsx
+++ b/docs/downloads/Subject Settings Matrix.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Subject Settings Matrix" sheetId="1" r:id="R1605a80ff87a4e7b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="C1-C3 Defaults" sheetId="2" r:id="R300ecaccc8284d70"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Subject Settings Matrix" sheetId="1" r:id="R2b71e983934b43cc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="C1-C3 Defaults" sheetId="2" r:id="R4c859fbab7294416"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -432,13 +432,13 @@
     <xdr:ext cx="24765000" cy="1200150"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="ef97ad79-dcc8-4f8a-bf02-5ad11eddf51a"/>
+        <xdr:cNvPr id="1" name="4e3c650b-177e-4591-96fd-6ce5c8637f71"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rf3c48f2783404676"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rd08045b2bc8648ef"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -5688,9 +5688,9 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing ns1:id="R3ce5f156e4b54536"/>
+  <x:drawing ns1:id="R667ec60e70704171"/>
   <x:tableParts count="1">
-    <x:tablePart ns1:id="R2edb6d31fea54b68"/>
+    <x:tablePart ns1:id="R6f4ec5d0f86f4607"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5725,7 +5725,7 @@
   <x:sheetData>
     <x:row r="1" ht="36" customHeight="1">
       <x:c r="A1" s="43" t="str">
-        <x:v>Approved registration targets pending physical verification. Ordinary copy/paste back to the matching C1–C3 column restores both the target values and compatible comparison highlighting.</x:v>
+        <x:v>Session-3 camera-body targets; lens Mode 1/3 remains pending. Edited targets require physical re-verification. Ordinary copy/paste back to the matching C1–C3 column restores both the target values and compatible comparison highlighting.</x:v>
       </x:c>
       <x:c r="B1" s="43"/>
       <x:c r="C1" s="43"/>
@@ -6812,7 +6812,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart ns1:id="Rc8c04f183a464052"/>
+    <x:tablePart ns1:id="R5430a6c1abbb482d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add lens-aware guidance and control references
</commit_message>
<xml_diff>
--- a/docs/downloads/Subject Settings Matrix.xlsx
+++ b/docs/downloads/Subject Settings Matrix.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Subject Settings Matrix" sheetId="1" r:id="R2b71e983934b43cc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="C1-C3 Defaults" sheetId="2" r:id="R4c859fbab7294416"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Subject Settings Matrix" sheetId="1" r:id="R4a02eb6137ad4a3a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="C1-C3 Defaults" sheetId="2" r:id="R7acf3d80f6c34912"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -432,13 +432,13 @@
     <xdr:ext cx="24765000" cy="1200150"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="4e3c650b-177e-4591-96fd-6ce5c8637f71"/>
+        <xdr:cNvPr id="1" name="5bb49d56-76b8-44d2-8c16-e921227b674f"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rd08045b2bc8648ef"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R385622037a8d4e94"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -5688,9 +5688,9 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing ns1:id="R667ec60e70704171"/>
+  <x:drawing ns1:id="Rd29f6c7ef03b4597"/>
   <x:tableParts count="1">
-    <x:tablePart ns1:id="R6f4ec5d0f86f4607"/>
+    <x:tablePart ns1:id="Raf616c98a43942cd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6812,7 +6812,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart ns1:id="R5430a6c1abbb482d"/>
+    <x:tablePart ns1:id="Rdbfd415a2e4d4840"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>